<commit_message>
Actualizar analisis de acciones
</commit_message>
<xml_diff>
--- a/analisis_acciones.xlsx
+++ b/analisis_acciones.xlsx
@@ -413,9 +413,442 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Accion</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Precio actual</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Probabilidad tecnica</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Entrada min</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Entrada max</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Stop loss</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Objetivo</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>RSI</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Riesgo</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Senal</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>220.42</v>
+      </c>
+      <c r="C2" t="n">
+        <v>85</v>
+      </c>
+      <c r="D2" t="n">
+        <v>217.11</v>
+      </c>
+      <c r="E2" t="n">
+        <v>222.62</v>
+      </c>
+      <c r="F2" t="n">
+        <v>209.4</v>
+      </c>
+      <c r="G2" t="n">
+        <v>238.05</v>
+      </c>
+      <c r="H2" t="n">
+        <v>2.23</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>MEDIO</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>POSIBLE COMPRA</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>458.83</v>
+      </c>
+      <c r="C3" t="n">
+        <v>85</v>
+      </c>
+      <c r="D3" t="n">
+        <v>451.95</v>
+      </c>
+      <c r="E3" t="n">
+        <v>463.42</v>
+      </c>
+      <c r="F3" t="n">
+        <v>435.89</v>
+      </c>
+      <c r="G3" t="n">
+        <v>495.54</v>
+      </c>
+      <c r="H3" t="n">
+        <v>4.36</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>ALTO</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>POSIBLE COMPRA</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>429.86</v>
+      </c>
+      <c r="C4" t="n">
+        <v>85</v>
+      </c>
+      <c r="D4" t="n">
+        <v>423.41</v>
+      </c>
+      <c r="E4" t="n">
+        <v>434.16</v>
+      </c>
+      <c r="F4" t="n">
+        <v>408.37</v>
+      </c>
+      <c r="G4" t="n">
+        <v>464.25</v>
+      </c>
+      <c r="H4" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>MEDIO</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>POSIBLE COMPRA</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>292.67</v>
+      </c>
+      <c r="C5" t="n">
+        <v>85</v>
+      </c>
+      <c r="D5" t="n">
+        <v>288.28</v>
+      </c>
+      <c r="E5" t="n">
+        <v>295.6</v>
+      </c>
+      <c r="F5" t="n">
+        <v>278.04</v>
+      </c>
+      <c r="G5" t="n">
+        <v>316.08</v>
+      </c>
+      <c r="H5" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>BAJO</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>POSIBLE COMPRA</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>421.45</v>
+      </c>
+      <c r="C6" t="n">
+        <v>85</v>
+      </c>
+      <c r="D6" t="n">
+        <v>415.13</v>
+      </c>
+      <c r="E6" t="n">
+        <v>425.66</v>
+      </c>
+      <c r="F6" t="n">
+        <v>400.38</v>
+      </c>
+      <c r="G6" t="n">
+        <v>455.17</v>
+      </c>
+      <c r="H6" t="n">
+        <v>2.47</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>MEDIO</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>POSIBLE COMPRA</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>394.42</v>
+      </c>
+      <c r="C7" t="n">
+        <v>85</v>
+      </c>
+      <c r="D7" t="n">
+        <v>388.5</v>
+      </c>
+      <c r="E7" t="n">
+        <v>398.36</v>
+      </c>
+      <c r="F7" t="n">
+        <v>374.69</v>
+      </c>
+      <c r="G7" t="n">
+        <v>425.97</v>
+      </c>
+      <c r="H7" t="n">
+        <v>1.93</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>BAJO</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>POSIBLE COMPRA</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>271.16</v>
+      </c>
+      <c r="C8" t="n">
+        <v>75</v>
+      </c>
+      <c r="D8" t="n">
+        <v>267.09</v>
+      </c>
+      <c r="E8" t="n">
+        <v>273.87</v>
+      </c>
+      <c r="F8" t="n">
+        <v>257.6</v>
+      </c>
+      <c r="G8" t="n">
+        <v>292.85</v>
+      </c>
+      <c r="H8" t="n">
+        <v>1.84</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>BAJO</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>POSIBLE COMPRA</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>409.38</v>
+      </c>
+      <c r="C9" t="n">
+        <v>65</v>
+      </c>
+      <c r="D9" t="n">
+        <v>403.23</v>
+      </c>
+      <c r="E9" t="n">
+        <v>413.47</v>
+      </c>
+      <c r="F9" t="n">
+        <v>388.91</v>
+      </c>
+      <c r="G9" t="n">
+        <v>442.13</v>
+      </c>
+      <c r="H9" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>BAJO</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>VIGILAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>600.84</v>
+      </c>
+      <c r="C10" t="n">
+        <v>65</v>
+      </c>
+      <c r="D10" t="n">
+        <v>591.83</v>
+      </c>
+      <c r="E10" t="n">
+        <v>606.85</v>
+      </c>
+      <c r="F10" t="n">
+        <v>570.8</v>
+      </c>
+      <c r="G10" t="n">
+        <v>648.91</v>
+      </c>
+      <c r="H10" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>MEDIO</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>VIGILAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>PLTR</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>134.79</v>
+      </c>
+      <c r="C11" t="n">
+        <v>50</v>
+      </c>
+      <c r="D11" t="n">
+        <v>132.76</v>
+      </c>
+      <c r="E11" t="n">
+        <v>136.13</v>
+      </c>
+      <c r="F11" t="n">
+        <v>128.05</v>
+      </c>
+      <c r="G11" t="n">
+        <v>145.57</v>
+      </c>
+      <c r="H11" t="n">
+        <v>3.26</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>MEDIO</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>NO COMPRAR</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>